<commit_message>
the chart and the table beneath it plotted different answers
Fixing the sensitivity table's basis and not the figure above it left the
picture on the book minority while the table under it read the adopted one
— the chart landing five to twenty pounds a share low against its own
table. The workbook's sensitivity sheet had the same shape with a further
twist: both its per-share columns took the book figure and only the second
said so, so a reader taking the unlabelled column for the study's answer
got a different one. Both now read the adopted basis and both say which.

The document said the minority is deducted "two different ways" in two
places and "three bases" in a third, while the summary table publishes
three columns. The count is now taken from the bases the study actually
carries, so it cannot disagree with the table it sits under.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017RcjXG4ETjADcoFJf123yY
</commit_message>
<xml_diff>
--- a/engine/tmgh_study/TMGH_Valuation_Model_02092026.xlsx
+++ b/engine/tmgh_study/TMGH_Valuation_Model_02092026.xlsx
@@ -2021,12 +2021,12 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Slower conversion, EGP/share</t>
+          <t>Slower conversion, EGP/share (minority at value share, adopted)</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Faster conversion, EGP/share (minority at book)</t>
+          <t>Faster conversion, EGP/share (minority at value share, adopted)</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -2040,10 +2040,10 @@
         <v>0.2437485685188716</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>211.95934597485</v>
+        <v>196.5101788932792</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>122.1265482723757</v>
+        <v>125.5209481014641</v>
       </c>
       <c r="D2" s="10">
         <f>B2/'Summary'!$B$2-1</f>
@@ -2055,10 +2055,10 @@
         <v>0.2837485685188716</v>
       </c>
       <c r="B3" s="9" t="n">
-        <v>152.3943501597619</v>
+        <v>149.4396952483696</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>70.10034183574056</v>
+        <v>84.40789729584293</v>
       </c>
       <c r="D3" s="10">
         <f>B3/'Summary'!$B$2-1</f>
@@ -2070,10 +2070,10 @@
         <v>0.3037485685188716</v>
       </c>
       <c r="B4" s="9" t="n">
-        <v>133.7027890895464</v>
+        <v>134.6689258121608</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>55.88696664744229</v>
+        <v>73.17595754356496</v>
       </c>
       <c r="D4" s="10">
         <f>B4/'Summary'!$B$2-1</f>
@@ -2085,10 +2085,10 @@
         <v>0.3237485685188716</v>
       </c>
       <c r="B5" s="9" t="n">
-        <v>118.9724199380305</v>
+        <v>123.028438127374</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>45.74742866171763</v>
+        <v>65.16331605181323</v>
       </c>
       <c r="D5" s="10">
         <f>B5/'Summary'!$B$2-1</f>
@@ -2100,10 +2100,10 @@
         <v>0.3437485685188716</v>
       </c>
       <c r="B6" s="9" t="n">
-        <v>107.0313026377783</v>
+        <v>113.5921213965149</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>38.35305553607058</v>
+        <v>59.32000632749752</v>
       </c>
       <c r="D6" s="10">
         <f>B6/'Summary'!$B$2-1</f>
@@ -2115,10 +2115,10 @@
         <v>0.3637485685188716</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>97.14815921409972</v>
+        <v>105.782092460582</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>32.8732712141484</v>
+        <v>54.98967616003811</v>
       </c>
       <c r="D7" s="10">
         <f>B7/'Summary'!$B$2-1</f>
@@ -2130,10 +2130,10 @@
         <v>0.4037485685188716</v>
       </c>
       <c r="B8" s="9" t="n">
-        <v>81.75426375262785</v>
+        <v>93.61726151188044</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>25.64354362310214</v>
+        <v>49.27647548446123</v>
       </c>
       <c r="D8" s="10">
         <f>B8/'Summary'!$B$2-1</f>

</xml_diff>